<commit_message>
Add QR generation and seat/BU support
Adds per-participant QR PNG generation and end-to-end support for seat_no and BU fields.
</commit_message>
<xml_diff>
--- a/tests/sample_data/2025-07-10 CDCS-Masterlist.xlsx
+++ b/tests/sample_data/2025-07-10 CDCS-Masterlist.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Wei Xian\Desktop\projects\msspc\tests\sample_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83826AFD-12FD-4715-9DDF-2468C8D051D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06917AD4-E105-4810-8F27-D318E13A7414}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="10875" yWindow="-15735" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Corporate" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="27">
   <si>
     <t>Name</t>
   </si>
@@ -98,6 +98,9 @@
   </si>
   <si>
     <t>Unique QR ID</t>
+  </si>
+  <si>
+    <t>Seat No</t>
   </si>
 </sst>
 </file>
@@ -505,7 +508,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E49"/>
+  <dimension ref="A1:F49"/>
   <sheetFormatPr defaultColWidth="42.109375" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11.77734375" bestFit="1" customWidth="1"/>
@@ -515,7 +518,7 @@
     <col min="5" max="5" width="5.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>25</v>
       </c>
@@ -531,10 +534,13 @@
       <c r="E1" s="4" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="F1" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2">
-        <v>1</v>
+        <v>750001</v>
       </c>
       <c r="B2" s="10" t="s">
         <v>3</v>
@@ -548,10 +554,13 @@
       <c r="E2" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="F2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3">
-        <v>2</v>
+        <v>750002</v>
       </c>
       <c r="B3" s="5" t="s">
         <v>6</v>
@@ -565,10 +574,13 @@
       <c r="E3" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="F3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4">
-        <v>3</v>
+        <v>750003</v>
       </c>
       <c r="B4" s="5" t="s">
         <v>19</v>
@@ -582,10 +594,13 @@
       <c r="E4" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="F4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5">
-        <v>4</v>
+        <v>750004</v>
       </c>
       <c r="B5" t="s">
         <v>21</v>
@@ -599,10 +614,13 @@
       <c r="E5" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="F5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6">
-        <v>5</v>
+        <v>750005</v>
       </c>
       <c r="B6" s="5" t="s">
         <v>9</v>
@@ -616,10 +634,13 @@
       <c r="E6" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="7" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="F6">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7">
-        <v>6</v>
+        <v>750006</v>
       </c>
       <c r="B7" s="5" t="s">
         <v>17</v>
@@ -633,10 +654,13 @@
       <c r="E7" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="F7">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8">
-        <v>7</v>
+        <v>750007</v>
       </c>
       <c r="B8" t="s">
         <v>15</v>
@@ -650,10 +674,13 @@
       <c r="E8" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="9" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="F8">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9">
-        <v>8</v>
+        <v>750008</v>
       </c>
       <c r="B9" s="5" t="s">
         <v>11</v>
@@ -667,10 +694,13 @@
       <c r="E9" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="10" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="F9">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10">
-        <v>9</v>
+        <v>750009</v>
       </c>
       <c r="B10" s="5" t="s">
         <v>13</v>
@@ -684,10 +714,13 @@
       <c r="E10" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="11" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="F10">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11">
-        <v>10</v>
+        <v>750010</v>
       </c>
       <c r="B11" t="s">
         <v>16</v>
@@ -701,28 +734,31 @@
       <c r="E11" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="12" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="F11">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B12" s="5"/>
       <c r="C12" s="6"/>
       <c r="D12" s="8"/>
     </row>
-    <row r="13" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B13" s="5"/>
       <c r="C13" s="6"/>
       <c r="D13" s="8"/>
     </row>
-    <row r="14" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B14" s="5"/>
       <c r="C14" s="6"/>
       <c r="D14" s="8"/>
     </row>
-    <row r="15" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B15" s="5"/>
       <c r="C15" s="9"/>
       <c r="D15" s="8"/>
     </row>
-    <row r="16" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B16" s="5"/>
       <c r="C16" s="6"/>
       <c r="D16" s="8"/>

</xml_diff>